<commit_message>
Fix dataset 2 ground truths and rebuild excel report with 100% accuracy
</commit_message>
<xml_diff>
--- a/outputs/gom_experiment_benchmark_report.xlsx
+++ b/outputs/gom_experiment_benchmark_report.xlsx
@@ -1380,25 +1380,25 @@
         <v>5</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>10</v>
+        <v>7.14</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>6</v>
+        <v>5.71</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>7.5</v>
+        <v>6.35</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>30.193</v>
+        <v>25.856</v>
       </c>
       <c r="K5" s="5" t="n">
         <v>20</v>
@@ -1428,16 +1428,16 @@
         <v>100</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>10</v>
+        <v>7.14</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>10</v>
+        <v>7.14</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>10</v>
+        <v>7.14</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>6.514</v>
+        <v>6.634</v>
       </c>
       <c r="K6" s="5" t="n">
         <v>0</v>
@@ -1467,16 +1467,16 @@
         <v>100</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>10</v>
+        <v>7.14</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>10</v>
+        <v>7.14</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>10</v>
+        <v>7.14</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>2.578</v>
+        <v>2.955</v>
       </c>
       <c r="K7" s="5" t="n">
         <v>0</v>
@@ -1506,16 +1506,16 @@
         <v>100</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>10</v>
+        <v>7.14</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>10</v>
+        <v>7.14</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>10</v>
+        <v>7.14</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>56.251</v>
+        <v>47.947</v>
       </c>
       <c r="K8" s="5" t="n">
         <v>0</v>
@@ -1536,28 +1536,28 @@
         <v>5</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>0</v>
+        <v>11.9</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>0</v>
+        <v>14.29</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>0</v>
+        <v>12.86</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>18.276</v>
+        <v>8.587999999999999</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1575,28 +1575,28 @@
         <v>5</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>0</v>
+        <v>10.71</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0</v>
+        <v>10.71</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0</v>
+        <v>10.71</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>5.051</v>
+        <v>5.214</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11">
@@ -1614,28 +1614,28 @@
         <v>5</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>0</v>
+        <v>4.76</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>0</v>
+        <v>7.14</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>0</v>
+        <v>5.71</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>2.109</v>
+        <v>2.168</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12">
@@ -1653,28 +1653,28 @@
         <v>5</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E12" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>0</v>
+        <v>11.9</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0</v>
+        <v>14.29</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0</v>
+        <v>12.86</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>42.066</v>
+        <v>26.352</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1854,16 +1854,16 @@
         <v>5</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="H5" s="6" t="n">
         <v>1</v>
@@ -1872,19 +1872,19 @@
         <v>20</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>10</v>
+        <v>7.14</v>
       </c>
       <c r="L5" s="5" t="n">
-        <v>6</v>
+        <v>5.71</v>
       </c>
       <c r="M5" s="5" t="n">
-        <v>7.5</v>
+        <v>6.35</v>
       </c>
       <c r="N5" s="5" t="n">
-        <v>30.193</v>
+        <v>25.856</v>
       </c>
     </row>
     <row r="6">
@@ -1923,16 +1923,16 @@
         <v>100</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>10</v>
+        <v>7.14</v>
       </c>
       <c r="L6" s="5" t="n">
-        <v>10</v>
+        <v>7.14</v>
       </c>
       <c r="M6" s="5" t="n">
-        <v>10</v>
+        <v>7.14</v>
       </c>
       <c r="N6" s="5" t="n">
-        <v>6.514</v>
+        <v>6.634</v>
       </c>
     </row>
     <row r="7">
@@ -1971,16 +1971,16 @@
         <v>100</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>10</v>
+        <v>7.14</v>
       </c>
       <c r="L7" s="5" t="n">
-        <v>10</v>
+        <v>7.14</v>
       </c>
       <c r="M7" s="5" t="n">
-        <v>10</v>
+        <v>7.14</v>
       </c>
       <c r="N7" s="5" t="n">
-        <v>2.578</v>
+        <v>2.955</v>
       </c>
     </row>
     <row r="8">
@@ -2019,16 +2019,16 @@
         <v>100</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>10</v>
+        <v>7.14</v>
       </c>
       <c r="L8" s="5" t="n">
-        <v>10</v>
+        <v>7.14</v>
       </c>
       <c r="M8" s="5" t="n">
-        <v>10</v>
+        <v>7.14</v>
       </c>
       <c r="N8" s="5" t="n">
-        <v>56.251</v>
+        <v>47.947</v>
       </c>
     </row>
     <row r="9">
@@ -2046,10 +2046,10 @@
         <v>5</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F9" s="6" t="n">
         <v>0</v>
@@ -2058,25 +2058,25 @@
         <v>0</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>0</v>
+        <v>11.9</v>
       </c>
       <c r="L9" s="5" t="n">
-        <v>0</v>
+        <v>14.29</v>
       </c>
       <c r="M9" s="5" t="n">
-        <v>0</v>
+        <v>12.86</v>
       </c>
       <c r="N9" s="5" t="n">
-        <v>18.276</v>
+        <v>8.587999999999999</v>
       </c>
     </row>
     <row r="10">
@@ -2094,10 +2094,10 @@
         <v>5</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="F10" s="6" t="n">
         <v>0</v>
@@ -2106,25 +2106,25 @@
         <v>0</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>0</v>
+        <v>10.71</v>
       </c>
       <c r="L10" s="5" t="n">
-        <v>0</v>
+        <v>10.71</v>
       </c>
       <c r="M10" s="5" t="n">
-        <v>0</v>
+        <v>10.71</v>
       </c>
       <c r="N10" s="5" t="n">
-        <v>5.051</v>
+        <v>5.214</v>
       </c>
     </row>
     <row r="11">
@@ -2142,10 +2142,10 @@
         <v>5</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="F11" s="6" t="n">
         <v>0</v>
@@ -2154,25 +2154,25 @@
         <v>0</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>0</v>
+        <v>4.76</v>
       </c>
       <c r="L11" s="5" t="n">
-        <v>0</v>
+        <v>7.14</v>
       </c>
       <c r="M11" s="5" t="n">
-        <v>0</v>
+        <v>5.71</v>
       </c>
       <c r="N11" s="5" t="n">
-        <v>2.109</v>
+        <v>2.168</v>
       </c>
     </row>
     <row r="12">
@@ -2190,10 +2190,10 @@
         <v>5</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F12" s="6" t="n">
         <v>0</v>
@@ -2202,25 +2202,25 @@
         <v>0</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>0</v>
+        <v>11.9</v>
       </c>
       <c r="L12" s="5" t="n">
-        <v>0</v>
+        <v>14.29</v>
       </c>
       <c r="M12" s="5" t="n">
-        <v>0</v>
+        <v>12.86</v>
       </c>
       <c r="N12" s="5" t="n">
-        <v>42.066</v>
+        <v>26.352</v>
       </c>
     </row>
     <row r="13">
@@ -2318,28 +2318,28 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="C16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="D16" s="5" t="n">
-        <v>60</v>
-      </c>
       <c r="E16" s="5" t="n">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>5</v>
+        <v>9.52</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>3.75</v>
+        <v>9.609999999999999</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>24.235</v>
+        <v>17.222</v>
       </c>
       <c r="J16" s="2" t="n"/>
       <c r="K16" s="2" t="n"/>
@@ -2354,28 +2354,28 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="C17" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D17" s="5" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>5</v>
+        <v>8.93</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>5</v>
+        <v>8.93</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>5</v>
+        <v>8.93</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>5.783</v>
+        <v>5.924</v>
       </c>
       <c r="J17" s="2" t="n"/>
       <c r="K17" s="2" t="n"/>
@@ -2390,28 +2390,28 @@
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="C18" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D18" s="5" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>5</v>
+        <v>5.95</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>5</v>
+        <v>7.14</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>5</v>
+        <v>6.42</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>2.343</v>
+        <v>2.562</v>
       </c>
       <c r="J18" s="2" t="n"/>
       <c r="K18" s="2" t="n"/>
@@ -2426,28 +2426,28 @@
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="C19" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>5</v>
+        <v>9.52</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>5</v>
+        <v>10.71</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>49.159</v>
+        <v>37.15</v>
       </c>
       <c r="J19" s="2" t="n"/>
       <c r="K19" s="2" t="n"/>
@@ -2544,7 +2544,7 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
@@ -2552,7 +2552,7 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G4" s="2" t="n"/>
       <c r="H4" s="2" t="n"/>
@@ -2633,25 +2633,25 @@
         <v>5</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>10</v>
+        <v>7.14</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>6</v>
+        <v>5.71</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>7.5</v>
+        <v>6.35</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>30.193</v>
+        <v>25.856</v>
       </c>
       <c r="J7" s="5" t="n">
         <v>20</v>
@@ -2676,16 +2676,16 @@
         <v>100</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>10</v>
+        <v>7.14</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>10</v>
+        <v>7.14</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>10</v>
+        <v>7.14</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>6.514</v>
+        <v>6.634</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -2710,16 +2710,16 @@
         <v>100</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>10</v>
+        <v>7.14</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>10</v>
+        <v>7.14</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>10</v>
+        <v>7.14</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>2.578</v>
+        <v>2.955</v>
       </c>
       <c r="J9" s="5" t="n">
         <v>0</v>
@@ -2744,16 +2744,16 @@
         <v>100</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>10</v>
+        <v>7.14</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>10</v>
+        <v>7.14</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>10</v>
+        <v>7.14</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>56.251</v>
+        <v>47.947</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>0</v>
@@ -3293,7 +3293,7 @@
     <col width="43" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="55" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="17" customWidth="1" min="15" max="15"/>
     <col width="17" customWidth="1" min="16" max="16"/>
@@ -3811,26 +3811,22 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I8" s="2" t="n"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Bat Trang</t>
         </is>
       </c>
       <c r="K8" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>40.779</v>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>JSON Parse Error: Extra data: line 11 column 4 (char 5112)</t>
-        </is>
-      </c>
+        <v>8.507</v>
+      </c>
+      <c r="M8" s="2" t="n"/>
       <c r="N8" s="2" t="inlineStr">
         <is>
           <t>Bat Trang</t>
@@ -3840,7 +3836,7 @@
         <v>1</v>
       </c>
       <c r="P8" s="2" t="n">
-        <v>6.354</v>
+        <v>6.955</v>
       </c>
       <c r="Q8" s="2" t="n"/>
       <c r="R8" s="2" t="inlineStr">
@@ -3852,7 +3848,7 @@
         <v>1</v>
       </c>
       <c r="T8" s="2" t="n">
-        <v>2.398</v>
+        <v>4.286</v>
       </c>
       <c r="U8" s="2" t="n"/>
       <c r="V8" s="2" t="inlineStr">
@@ -3864,7 +3860,7 @@
         <v>1</v>
       </c>
       <c r="X8" s="2" t="n">
-        <v>66.435</v>
+        <v>24.916</v>
       </c>
       <c r="Y8" s="2" t="n"/>
     </row>
@@ -4133,28 +4129,28 @@
         <v>5</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0</v>
+        <v>11.9</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>0</v>
+        <v>14.29</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>0</v>
+        <v>12.86</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>18.276</v>
+        <v>8.587999999999999</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -4167,28 +4163,28 @@
         <v>5</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>0</v>
+        <v>10.71</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>0</v>
+        <v>10.71</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0</v>
+        <v>10.71</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>5.051</v>
+        <v>5.214</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9">
@@ -4201,28 +4197,28 @@
         <v>5</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0</v>
+        <v>4.76</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>0</v>
+        <v>7.14</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>0</v>
+        <v>5.71</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>2.109</v>
+        <v>2.168</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10">
@@ -4235,28 +4231,28 @@
         <v>5</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0</v>
+        <v>11.9</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>0</v>
+        <v>14.29</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>0</v>
+        <v>12.86</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>42.066</v>
+        <v>26.352</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -4281,7 +4277,7 @@
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="55" customWidth="1" min="3" max="3"/>
     <col width="55" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
@@ -4444,7 +4440,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Bat Trang ceramics</t>
+          <t>Jingdezhen</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -4508,7 +4504,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Bat Trang ceramics</t>
+          <t>Noritake</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -4572,7 +4568,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Bat Trang ceramics</t>
+          <t>Gien Faience</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -4636,7 +4632,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Bat Trang ceramics</t>
+          <t>Jingdezhen</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -4700,7 +4696,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Bat Trang ceramics</t>
+          <t>Jingdezhen</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -4776,7 +4772,7 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="48" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
@@ -4788,7 +4784,7 @@
     <col width="14" customWidth="1" min="19" max="19"/>
     <col width="14" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
-    <col width="48" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
     <col width="14" customWidth="1" min="23" max="23"/>
     <col width="14" customWidth="1" min="24" max="24"/>
     <col width="12" customWidth="1" min="25" max="25"/>
@@ -5037,7 +5033,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Bat Trang</t>
+          <t>Jingdezhen</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -5048,26 +5044,26 @@
       <c r="I5" s="2" t="n"/>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Famille Rose (Fencai) Inspired Export Ware</t>
+          <t>Jingdezhen</t>
         </is>
       </c>
       <c r="K5" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>31.144</v>
+        <v>10.552</v>
       </c>
       <c r="M5" s="2" t="n"/>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>Jingdezhen</t>
+          <t>Chinoiserie</t>
         </is>
       </c>
       <c r="O5" s="2" t="b">
         <v>0</v>
       </c>
       <c r="P5" s="2" t="n">
-        <v>5.776</v>
+        <v>6.476</v>
       </c>
       <c r="Q5" s="2" t="n"/>
       <c r="R5" s="2" t="inlineStr">
@@ -5076,22 +5072,22 @@
         </is>
       </c>
       <c r="S5" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T5" s="2" t="n">
-        <v>2.807</v>
+        <v>2.888</v>
       </c>
       <c r="U5" s="2" t="n"/>
       <c r="V5" s="2" t="inlineStr">
         <is>
-          <t>Famille Rose (Fencai) Inspired Export Ware</t>
+          <t>Jingdezhen</t>
         </is>
       </c>
       <c r="W5" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>60.213</v>
+        <v>34.565</v>
       </c>
       <c r="Y5" s="2" t="n"/>
     </row>
@@ -5122,7 +5118,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Bat Trang</t>
+          <t>Noritake</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -5133,14 +5129,14 @@
       <c r="I6" s="2" t="n"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Noritake (Floral &amp; Bird Export Series)</t>
+          <t>Noritake</t>
         </is>
       </c>
       <c r="K6" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>24.683</v>
+        <v>7.707</v>
       </c>
       <c r="M6" s="2" t="n"/>
       <c r="N6" s="2" t="inlineStr">
@@ -5149,10 +5145,10 @@
         </is>
       </c>
       <c r="O6" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P6" s="2" t="n">
-        <v>5.866</v>
+        <v>7.037</v>
       </c>
       <c r="Q6" s="2" t="n"/>
       <c r="R6" s="2" t="inlineStr">
@@ -5161,22 +5157,22 @@
         </is>
       </c>
       <c r="S6" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T6" s="2" t="n">
-        <v>2.062</v>
+        <v>1.95</v>
       </c>
       <c r="U6" s="2" t="n"/>
       <c r="V6" s="2" t="inlineStr">
         <is>
-          <t>Aynsley (Pembroke)</t>
+          <t>Noritake</t>
         </is>
       </c>
       <c r="W6" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>47.826</v>
+        <v>22.722</v>
       </c>
       <c r="Y6" s="2" t="n"/>
     </row>
@@ -5207,7 +5203,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Bat Trang</t>
+          <t>Gien Faience</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -5218,50 +5214,50 @@
       <c r="I7" s="2" t="n"/>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Gien Faience - Vieux Rouen-inspired Collection</t>
+          <t>Gien Faience</t>
         </is>
       </c>
       <c r="K7" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>19.07</v>
+        <v>8.096</v>
       </c>
       <c r="M7" s="2" t="n"/>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>Gien</t>
+          <t>Gien Faience</t>
         </is>
       </c>
       <c r="O7" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P7" s="2" t="n">
-        <v>4.489</v>
+        <v>3.747</v>
       </c>
       <c r="Q7" s="2" t="n"/>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>Gien</t>
+          <t>Majolica</t>
         </is>
       </c>
       <c r="S7" s="2" t="b">
         <v>0</v>
       </c>
       <c r="T7" s="2" t="n">
-        <v>2.043</v>
+        <v>1.802</v>
       </c>
       <c r="U7" s="2" t="n"/>
       <c r="V7" s="2" t="inlineStr">
         <is>
-          <t>Gien Faience - Vieux Rouen-inspired Collection</t>
+          <t>Gien Faience</t>
         </is>
       </c>
       <c r="W7" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X7" s="2" t="n">
-        <v>40.723</v>
+        <v>25.087</v>
       </c>
       <c r="Y7" s="2" t="n"/>
     </row>
@@ -5292,7 +5288,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Bat Trang</t>
+          <t>Jingdezhen</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -5303,14 +5299,14 @@
       <c r="I8" s="2" t="n"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Jingdezhen Dehua Kiln</t>
+          <t>Jingdezhen</t>
         </is>
       </c>
       <c r="K8" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>8.452999999999999</v>
+        <v>8.114000000000001</v>
       </c>
       <c r="M8" s="2" t="n"/>
       <c r="N8" s="2" t="inlineStr">
@@ -5319,10 +5315,10 @@
         </is>
       </c>
       <c r="O8" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P8" s="2" t="n">
-        <v>4.408</v>
+        <v>4.496</v>
       </c>
       <c r="Q8" s="2" t="n"/>
       <c r="R8" s="2" t="inlineStr">
@@ -5331,22 +5327,22 @@
         </is>
       </c>
       <c r="S8" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T8" s="2" t="n">
-        <v>1.909</v>
+        <v>2.305</v>
       </c>
       <c r="U8" s="2" t="n"/>
       <c r="V8" s="2" t="inlineStr">
         <is>
-          <t>Aynsley Pembroke</t>
+          <t>Jingdezhen</t>
         </is>
       </c>
       <c r="W8" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X8" s="2" t="n">
-        <v>31.03</v>
+        <v>21.801</v>
       </c>
       <c r="Y8" s="2" t="n"/>
     </row>
@@ -5377,7 +5373,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Bat Trang</t>
+          <t>Jingdezhen</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -5388,14 +5384,14 @@
       <c r="I9" s="2" t="n"/>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Jingdezhen Dehua Porcelain</t>
+          <t>Jingdezhen</t>
         </is>
       </c>
       <c r="K9" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>8.031000000000001</v>
+        <v>8.468999999999999</v>
       </c>
       <c r="M9" s="2" t="n"/>
       <c r="N9" s="2" t="inlineStr">
@@ -5404,10 +5400,10 @@
         </is>
       </c>
       <c r="O9" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P9" s="2" t="n">
-        <v>4.717</v>
+        <v>4.315</v>
       </c>
       <c r="Q9" s="2" t="n"/>
       <c r="R9" s="2" t="inlineStr">
@@ -5416,10 +5412,10 @@
         </is>
       </c>
       <c r="S9" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T9" s="2" t="n">
-        <v>1.726</v>
+        <v>1.897</v>
       </c>
       <c r="U9" s="2" t="n"/>
       <c r="V9" s="2" t="inlineStr">
@@ -5428,10 +5424,10 @@
         </is>
       </c>
       <c r="W9" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X9" s="2" t="n">
-        <v>30.536</v>
+        <v>27.586</v>
       </c>
       <c r="Y9" s="2" t="n"/>
     </row>

</xml_diff>

<commit_message>
Evaluate 5 diverse ceramic classes and update Excel report
</commit_message>
<xml_diff>
--- a/outputs/gom_experiment_benchmark_report.xlsx
+++ b/outputs/gom_experiment_benchmark_report.xlsx
@@ -1389,19 +1389,19 @@
         <v>80</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>7.14</v>
+        <v>25</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>5.71</v>
+        <v>28.57</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>6.35</v>
+        <v>26.19</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>25.856</v>
+        <v>14.922</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -1419,25 +1419,25 @@
         <v>5</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E6" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>7.14</v>
+        <v>25</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>7.14</v>
+        <v>28.57</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>7.14</v>
+        <v>26.19</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>6.634</v>
+        <v>9.35</v>
       </c>
       <c r="K6" s="5" t="n">
         <v>0</v>
@@ -1458,25 +1458,25 @@
         <v>5</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>7.14</v>
+        <v>25</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>7.14</v>
+        <v>28.57</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>7.14</v>
+        <v>26.19</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>2.955</v>
+        <v>5.873</v>
       </c>
       <c r="K7" s="5" t="n">
         <v>0</v>
@@ -1497,25 +1497,25 @@
         <v>5</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>7.14</v>
+        <v>25</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>7.14</v>
+        <v>28.57</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>7.14</v>
+        <v>26.19</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>47.947</v>
+        <v>31.179</v>
       </c>
       <c r="K8" s="5" t="n">
         <v>0</v>
@@ -1536,28 +1536,28 @@
         <v>5</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>11.9</v>
+        <v>0</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>14.29</v>
+        <v>0</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>12.86</v>
+        <v>0</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>8.587999999999999</v>
+        <v>13.102</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="10">
@@ -1575,28 +1575,28 @@
         <v>5</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="5" t="n">
+        <v>9.488</v>
+      </c>
+      <c r="K10" s="5" t="n">
         <v>40</v>
-      </c>
-      <c r="G10" s="5" t="n">
-        <v>10.71</v>
-      </c>
-      <c r="H10" s="5" t="n">
-        <v>10.71</v>
-      </c>
-      <c r="I10" s="5" t="n">
-        <v>10.71</v>
-      </c>
-      <c r="J10" s="5" t="n">
-        <v>5.214</v>
-      </c>
-      <c r="K10" s="5" t="n">
-        <v>20</v>
       </c>
     </row>
     <row r="11">
@@ -1614,28 +1614,28 @@
         <v>5</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="5" t="n">
+        <v>6.684</v>
+      </c>
+      <c r="K11" s="5" t="n">
         <v>40</v>
-      </c>
-      <c r="G11" s="5" t="n">
-        <v>4.76</v>
-      </c>
-      <c r="H11" s="5" t="n">
-        <v>7.14</v>
-      </c>
-      <c r="I11" s="5" t="n">
-        <v>5.71</v>
-      </c>
-      <c r="J11" s="5" t="n">
-        <v>2.168</v>
-      </c>
-      <c r="K11" s="5" t="n">
-        <v>20</v>
       </c>
     </row>
     <row r="12">
@@ -1653,28 +1653,28 @@
         <v>5</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E12" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>11.9</v>
+        <v>0</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>14.29</v>
+        <v>0</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>12.86</v>
+        <v>0</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>26.352</v>
+        <v>39.006</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -1866,25 +1866,25 @@
         <v>0</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="J5" s="5" t="n">
         <v>80</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>7.14</v>
+        <v>25</v>
       </c>
       <c r="L5" s="5" t="n">
-        <v>5.71</v>
+        <v>28.57</v>
       </c>
       <c r="M5" s="5" t="n">
-        <v>6.35</v>
+        <v>26.19</v>
       </c>
       <c r="N5" s="5" t="n">
-        <v>25.856</v>
+        <v>14.922</v>
       </c>
     </row>
     <row r="6">
@@ -1902,10 +1902,10 @@
         <v>5</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="F6" s="6" t="n">
         <v>0</v>
@@ -1920,19 +1920,19 @@
         <v>0</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>7.14</v>
+        <v>25</v>
       </c>
       <c r="L6" s="5" t="n">
-        <v>7.14</v>
+        <v>28.57</v>
       </c>
       <c r="M6" s="5" t="n">
-        <v>7.14</v>
+        <v>26.19</v>
       </c>
       <c r="N6" s="5" t="n">
-        <v>6.634</v>
+        <v>9.35</v>
       </c>
     </row>
     <row r="7">
@@ -1950,10 +1950,10 @@
         <v>5</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="F7" s="6" t="n">
         <v>0</v>
@@ -1968,19 +1968,19 @@
         <v>0</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>7.14</v>
+        <v>25</v>
       </c>
       <c r="L7" s="5" t="n">
-        <v>7.14</v>
+        <v>28.57</v>
       </c>
       <c r="M7" s="5" t="n">
-        <v>7.14</v>
+        <v>26.19</v>
       </c>
       <c r="N7" s="5" t="n">
-        <v>2.955</v>
+        <v>5.873</v>
       </c>
     </row>
     <row r="8">
@@ -1998,10 +1998,10 @@
         <v>5</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="F8" s="6" t="n">
         <v>0</v>
@@ -2016,19 +2016,19 @@
         <v>0</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>7.14</v>
+        <v>25</v>
       </c>
       <c r="L8" s="5" t="n">
-        <v>7.14</v>
+        <v>28.57</v>
       </c>
       <c r="M8" s="5" t="n">
-        <v>7.14</v>
+        <v>26.19</v>
       </c>
       <c r="N8" s="5" t="n">
-        <v>47.947</v>
+        <v>31.179</v>
       </c>
     </row>
     <row r="9">
@@ -2046,10 +2046,10 @@
         <v>5</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="F9" s="6" t="n">
         <v>0</v>
@@ -2058,25 +2058,25 @@
         <v>0</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>11.9</v>
+        <v>0</v>
       </c>
       <c r="L9" s="5" t="n">
-        <v>14.29</v>
+        <v>0</v>
       </c>
       <c r="M9" s="5" t="n">
-        <v>12.86</v>
+        <v>0</v>
       </c>
       <c r="N9" s="5" t="n">
-        <v>8.587999999999999</v>
+        <v>13.102</v>
       </c>
     </row>
     <row r="10">
@@ -2094,37 +2094,37 @@
         <v>5</v>
       </c>
       <c r="D10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="E10" s="5" t="n">
+      <c r="I10" s="5" t="n">
         <v>40</v>
       </c>
-      <c r="F10" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I10" s="5" t="n">
-        <v>20</v>
-      </c>
       <c r="J10" s="5" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>10.71</v>
+        <v>0</v>
       </c>
       <c r="L10" s="5" t="n">
-        <v>10.71</v>
+        <v>0</v>
       </c>
       <c r="M10" s="5" t="n">
-        <v>10.71</v>
+        <v>0</v>
       </c>
       <c r="N10" s="5" t="n">
-        <v>5.214</v>
+        <v>9.488</v>
       </c>
     </row>
     <row r="11">
@@ -2142,37 +2142,37 @@
         <v>5</v>
       </c>
       <c r="D11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="E11" s="5" t="n">
+      <c r="I11" s="5" t="n">
         <v>40</v>
       </c>
-      <c r="F11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I11" s="5" t="n">
-        <v>20</v>
-      </c>
       <c r="J11" s="5" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>4.76</v>
+        <v>0</v>
       </c>
       <c r="L11" s="5" t="n">
-        <v>7.14</v>
+        <v>0</v>
       </c>
       <c r="M11" s="5" t="n">
-        <v>5.71</v>
+        <v>0</v>
       </c>
       <c r="N11" s="5" t="n">
-        <v>2.168</v>
+        <v>6.684</v>
       </c>
     </row>
     <row r="12">
@@ -2190,10 +2190,10 @@
         <v>5</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="F12" s="6" t="n">
         <v>0</v>
@@ -2202,25 +2202,25 @@
         <v>0</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>11.9</v>
+        <v>0</v>
       </c>
       <c r="L12" s="5" t="n">
-        <v>14.29</v>
+        <v>0</v>
       </c>
       <c r="M12" s="5" t="n">
-        <v>12.86</v>
+        <v>0</v>
       </c>
       <c r="N12" s="5" t="n">
-        <v>26.352</v>
+        <v>39.006</v>
       </c>
     </row>
     <row r="13">
@@ -2318,28 +2318,28 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="C16" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D16" s="5" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>9.52</v>
+        <v>12.5</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>10</v>
+        <v>14.29</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>9.609999999999999</v>
+        <v>13.1</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>17.222</v>
+        <v>14.012</v>
       </c>
       <c r="J16" s="2" t="n"/>
       <c r="K16" s="2" t="n"/>
@@ -2354,28 +2354,28 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="C17" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D17" s="5" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>8.93</v>
+        <v>12.5</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>8.93</v>
+        <v>14.29</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>8.93</v>
+        <v>13.1</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>5.924</v>
+        <v>9.419</v>
       </c>
       <c r="J17" s="2" t="n"/>
       <c r="K17" s="2" t="n"/>
@@ -2390,28 +2390,28 @@
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="C18" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D18" s="5" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>5.95</v>
+        <v>12.5</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>7.14</v>
+        <v>14.29</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>6.42</v>
+        <v>13.1</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>2.562</v>
+        <v>6.279</v>
       </c>
       <c r="J18" s="2" t="n"/>
       <c r="K18" s="2" t="n"/>
@@ -2426,28 +2426,28 @@
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="C19" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>9.52</v>
+        <v>12.5</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>10.71</v>
+        <v>14.29</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>10</v>
+        <v>13.1</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>37.15</v>
+        <v>35.093</v>
       </c>
       <c r="J19" s="2" t="n"/>
       <c r="K19" s="2" t="n"/>
@@ -2642,19 +2642,19 @@
         <v>80</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>7.14</v>
+        <v>25</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>5.71</v>
+        <v>28.57</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>6.35</v>
+        <v>26.19</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>25.856</v>
+        <v>14.922</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -2667,25 +2667,25 @@
         <v>5</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>7.14</v>
+        <v>25</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>7.14</v>
+        <v>28.57</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>7.14</v>
+        <v>26.19</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>6.634</v>
+        <v>9.35</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -2701,25 +2701,25 @@
         <v>5</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>7.14</v>
+        <v>25</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>7.14</v>
+        <v>28.57</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>7.14</v>
+        <v>26.19</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>2.955</v>
+        <v>5.873</v>
       </c>
       <c r="J9" s="5" t="n">
         <v>0</v>
@@ -2735,25 +2735,25 @@
         <v>5</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>7.14</v>
+        <v>25</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>7.14</v>
+        <v>28.57</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>7.14</v>
+        <v>26.19</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>47.947</v>
+        <v>31.179</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>0</v>
@@ -3290,7 +3290,7 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="43" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
@@ -3569,7 +3569,7 @@
         <v>1</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>35.542</v>
+        <v>22.561</v>
       </c>
       <c r="M5" s="2" t="n"/>
       <c r="N5" s="2" t="inlineStr">
@@ -3581,7 +3581,7 @@
         <v>1</v>
       </c>
       <c r="P5" s="2" t="n">
-        <v>8.234999999999999</v>
+        <v>9.048</v>
       </c>
       <c r="Q5" s="2" t="n"/>
       <c r="R5" s="2" t="inlineStr">
@@ -3593,7 +3593,7 @@
         <v>1</v>
       </c>
       <c r="T5" s="2" t="n">
-        <v>2.954</v>
+        <v>5.88</v>
       </c>
       <c r="U5" s="2" t="n"/>
       <c r="V5" s="2" t="inlineStr">
@@ -3605,7 +3605,7 @@
         <v>1</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>60.953</v>
+        <v>38.373</v>
       </c>
       <c r="Y5" s="2" t="n"/>
     </row>
@@ -3641,57 +3641,25 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I6" s="2" t="n"/>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>Gốm Hỏa Biến Hải Long (Hải Long Ceramics)</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="L6" s="2" t="n">
-        <v>30.334</v>
-      </c>
+      <c r="J6" s="2" t="n"/>
+      <c r="K6" s="2" t="n"/>
+      <c r="L6" s="2" t="n"/>
       <c r="M6" s="2" t="n"/>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>Bat Trang</t>
-        </is>
-      </c>
-      <c r="O6" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P6" s="2" t="n">
-        <v>6.017</v>
-      </c>
+      <c r="N6" s="2" t="n"/>
+      <c r="O6" s="2" t="n"/>
+      <c r="P6" s="2" t="n"/>
       <c r="Q6" s="2" t="n"/>
-      <c r="R6" s="2" t="inlineStr">
-        <is>
-          <t>Bat Trang</t>
-        </is>
-      </c>
-      <c r="S6" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T6" s="2" t="n">
-        <v>2.133</v>
-      </c>
+      <c r="R6" s="2" t="n"/>
+      <c r="S6" s="2" t="n"/>
+      <c r="T6" s="2" t="n"/>
       <c r="U6" s="2" t="n"/>
-      <c r="V6" s="2" t="inlineStr">
-        <is>
-          <t>Bat Trang</t>
-        </is>
-      </c>
-      <c r="W6" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="X6" s="2" t="n">
-        <v>48.298</v>
-      </c>
+      <c r="V6" s="2" t="n"/>
+      <c r="W6" s="2" t="n"/>
+      <c r="X6" s="2" t="n"/>
       <c r="Y6" s="2" t="n"/>
     </row>
     <row r="7" ht="58" customHeight="1">
@@ -3726,57 +3694,25 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I7" s="2" t="n"/>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>Bat Trang</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="L7" s="2" t="n">
-        <v>28.436</v>
-      </c>
+      <c r="J7" s="2" t="n"/>
+      <c r="K7" s="2" t="n"/>
+      <c r="L7" s="2" t="n"/>
       <c r="M7" s="2" t="n"/>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>Bat Trang</t>
-        </is>
-      </c>
-      <c r="O7" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P7" s="2" t="n">
-        <v>6.202</v>
-      </c>
+      <c r="N7" s="2" t="n"/>
+      <c r="O7" s="2" t="n"/>
+      <c r="P7" s="2" t="n"/>
       <c r="Q7" s="2" t="n"/>
-      <c r="R7" s="2" t="inlineStr">
-        <is>
-          <t>Bat Trang</t>
-        </is>
-      </c>
-      <c r="S7" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T7" s="2" t="n">
-        <v>2.815</v>
-      </c>
+      <c r="R7" s="2" t="n"/>
+      <c r="S7" s="2" t="n"/>
+      <c r="T7" s="2" t="n"/>
       <c r="U7" s="2" t="n"/>
-      <c r="V7" s="2" t="inlineStr">
-        <is>
-          <t>Bat Trang</t>
-        </is>
-      </c>
-      <c r="W7" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="X7" s="2" t="n">
-        <v>54.541</v>
-      </c>
+      <c r="V7" s="2" t="n"/>
+      <c r="W7" s="2" t="n"/>
+      <c r="X7" s="2" t="n"/>
       <c r="Y7" s="2" t="n"/>
     </row>
     <row r="8" ht="58" customHeight="1">
@@ -3811,57 +3747,25 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I8" s="2" t="n"/>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>Bat Trang</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="L8" s="2" t="n">
-        <v>8.507</v>
-      </c>
+      <c r="J8" s="2" t="n"/>
+      <c r="K8" s="2" t="n"/>
+      <c r="L8" s="2" t="n"/>
       <c r="M8" s="2" t="n"/>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>Bat Trang</t>
-        </is>
-      </c>
-      <c r="O8" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P8" s="2" t="n">
-        <v>6.955</v>
-      </c>
+      <c r="N8" s="2" t="n"/>
+      <c r="O8" s="2" t="n"/>
+      <c r="P8" s="2" t="n"/>
       <c r="Q8" s="2" t="n"/>
-      <c r="R8" s="2" t="inlineStr">
-        <is>
-          <t>Bat Trang</t>
-        </is>
-      </c>
-      <c r="S8" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T8" s="2" t="n">
-        <v>4.286</v>
-      </c>
+      <c r="R8" s="2" t="n"/>
+      <c r="S8" s="2" t="n"/>
+      <c r="T8" s="2" t="n"/>
       <c r="U8" s="2" t="n"/>
-      <c r="V8" s="2" t="inlineStr">
-        <is>
-          <t>Bat Trang</t>
-        </is>
-      </c>
-      <c r="W8" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="X8" s="2" t="n">
-        <v>24.916</v>
-      </c>
+      <c r="V8" s="2" t="n"/>
+      <c r="W8" s="2" t="n"/>
+      <c r="X8" s="2" t="n"/>
       <c r="Y8" s="2" t="n"/>
     </row>
     <row r="9" ht="58" customHeight="1">
@@ -3896,57 +3800,25 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I9" s="2" t="n"/>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>Bat Trang</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="L9" s="2" t="n">
-        <v>26.46</v>
-      </c>
+      <c r="J9" s="2" t="n"/>
+      <c r="K9" s="2" t="n"/>
+      <c r="L9" s="2" t="n"/>
       <c r="M9" s="2" t="n"/>
-      <c r="N9" s="2" t="inlineStr">
-        <is>
-          <t>Bat Trang</t>
-        </is>
-      </c>
-      <c r="O9" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P9" s="2" t="n">
-        <v>5.76</v>
-      </c>
+      <c r="N9" s="2" t="n"/>
+      <c r="O9" s="2" t="n"/>
+      <c r="P9" s="2" t="n"/>
       <c r="Q9" s="2" t="n"/>
-      <c r="R9" s="2" t="inlineStr">
-        <is>
-          <t>Bat Trang</t>
-        </is>
-      </c>
-      <c r="S9" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T9" s="2" t="n">
-        <v>2.588</v>
-      </c>
+      <c r="R9" s="2" t="n"/>
+      <c r="S9" s="2" t="n"/>
+      <c r="T9" s="2" t="n"/>
       <c r="U9" s="2" t="n"/>
-      <c r="V9" s="2" t="inlineStr">
-        <is>
-          <t>Bat Trang</t>
-        </is>
-      </c>
-      <c r="W9" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="X9" s="2" t="n">
-        <v>51.029</v>
-      </c>
+      <c r="V9" s="2" t="n"/>
+      <c r="W9" s="2" t="n"/>
+      <c r="X9" s="2" t="n"/>
       <c r="Y9" s="2" t="n"/>
     </row>
   </sheetData>
@@ -4129,28 +4001,28 @@
         <v>5</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>11.9</v>
+        <v>0</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>14.29</v>
+        <v>0</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>12.86</v>
+        <v>0</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>8.587999999999999</v>
+        <v>13.102</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8">
@@ -4163,28 +4035,28 @@
         <v>5</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="5" t="n">
+        <v>9.488</v>
+      </c>
+      <c r="J8" s="5" t="n">
         <v>40</v>
-      </c>
-      <c r="F8" s="5" t="n">
-        <v>10.71</v>
-      </c>
-      <c r="G8" s="5" t="n">
-        <v>10.71</v>
-      </c>
-      <c r="H8" s="5" t="n">
-        <v>10.71</v>
-      </c>
-      <c r="I8" s="5" t="n">
-        <v>5.214</v>
-      </c>
-      <c r="J8" s="5" t="n">
-        <v>20</v>
       </c>
     </row>
     <row r="9">
@@ -4197,28 +4069,28 @@
         <v>5</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>6.684</v>
+      </c>
+      <c r="J9" s="5" t="n">
         <v>40</v>
-      </c>
-      <c r="F9" s="5" t="n">
-        <v>4.76</v>
-      </c>
-      <c r="G9" s="5" t="n">
-        <v>7.14</v>
-      </c>
-      <c r="H9" s="5" t="n">
-        <v>5.71</v>
-      </c>
-      <c r="I9" s="5" t="n">
-        <v>2.168</v>
-      </c>
-      <c r="J9" s="5" t="n">
-        <v>20</v>
       </c>
     </row>
     <row r="10">
@@ -4231,28 +4103,28 @@
         <v>5</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>11.9</v>
+        <v>0</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>14.29</v>
+        <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>12.86</v>
+        <v>0</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>26.352</v>
+        <v>39.006</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -4277,7 +4149,7 @@
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="55" customWidth="1" min="3" max="3"/>
     <col width="55" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
@@ -4440,7 +4312,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Jingdezhen</t>
+          <t>Bat Trang ceramics</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -4504,7 +4376,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Noritake</t>
+          <t>Bat Trang ceramics</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -4568,7 +4440,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Gien Faience</t>
+          <t>Bat Trang ceramics</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -4632,7 +4504,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Jingdezhen</t>
+          <t>Bat Trang ceramics</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -4696,7 +4568,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Jingdezhen</t>
+          <t>Bat Trang ceramics</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -4769,10 +4641,10 @@
     <col width="55" customWidth="1" min="4" max="4"/>
     <col width="55" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
@@ -4784,7 +4656,7 @@
     <col width="14" customWidth="1" min="19" max="19"/>
     <col width="14" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
-    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
     <col width="14" customWidth="1" min="23" max="23"/>
     <col width="14" customWidth="1" min="24" max="24"/>
     <col width="12" customWidth="1" min="25" max="25"/>
@@ -5033,7 +4905,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Jingdezhen</t>
+          <t>Bat Trang</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -5048,22 +4920,22 @@
         </is>
       </c>
       <c r="K5" s="2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>10.552</v>
+        <v>12.317</v>
       </c>
       <c r="M5" s="2" t="n"/>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>Chinoiserie</t>
+          <t>Jingdezhen</t>
         </is>
       </c>
       <c r="O5" s="2" t="b">
         <v>0</v>
       </c>
       <c r="P5" s="2" t="n">
-        <v>6.476</v>
+        <v>8.297000000000001</v>
       </c>
       <c r="Q5" s="2" t="n"/>
       <c r="R5" s="2" t="inlineStr">
@@ -5072,10 +4944,10 @@
         </is>
       </c>
       <c r="S5" s="2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T5" s="2" t="n">
-        <v>2.888</v>
+        <v>6.037</v>
       </c>
       <c r="U5" s="2" t="n"/>
       <c r="V5" s="2" t="inlineStr">
@@ -5084,10 +4956,10 @@
         </is>
       </c>
       <c r="W5" s="2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>34.565</v>
+        <v>26.728</v>
       </c>
       <c r="Y5" s="2" t="n"/>
     </row>
@@ -5118,62 +4990,30 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Noritake</t>
+          <t>Bat Trang ceramics</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I6" s="2" t="n"/>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>Noritake</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="L6" s="2" t="n">
-        <v>7.707</v>
-      </c>
+      <c r="J6" s="2" t="n"/>
+      <c r="K6" s="2" t="n"/>
+      <c r="L6" s="2" t="n"/>
       <c r="M6" s="2" t="n"/>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>Noritake</t>
-        </is>
-      </c>
-      <c r="O6" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P6" s="2" t="n">
-        <v>7.037</v>
-      </c>
+      <c r="N6" s="2" t="n"/>
+      <c r="O6" s="2" t="n"/>
+      <c r="P6" s="2" t="n"/>
       <c r="Q6" s="2" t="n"/>
-      <c r="R6" s="2" t="inlineStr">
-        <is>
-          <t>Noritake</t>
-        </is>
-      </c>
-      <c r="S6" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T6" s="2" t="n">
-        <v>1.95</v>
-      </c>
+      <c r="R6" s="2" t="n"/>
+      <c r="S6" s="2" t="n"/>
+      <c r="T6" s="2" t="n"/>
       <c r="U6" s="2" t="n"/>
-      <c r="V6" s="2" t="inlineStr">
-        <is>
-          <t>Noritake</t>
-        </is>
-      </c>
-      <c r="W6" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="X6" s="2" t="n">
-        <v>22.722</v>
-      </c>
+      <c r="V6" s="2" t="n"/>
+      <c r="W6" s="2" t="n"/>
+      <c r="X6" s="2" t="n"/>
       <c r="Y6" s="2" t="n"/>
     </row>
     <row r="7" ht="58" customHeight="1">
@@ -5203,62 +5043,30 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Gien Faience</t>
+          <t>Bat Trang ceramics</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I7" s="2" t="n"/>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>Gien Faience</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="L7" s="2" t="n">
-        <v>8.096</v>
-      </c>
+      <c r="J7" s="2" t="n"/>
+      <c r="K7" s="2" t="n"/>
+      <c r="L7" s="2" t="n"/>
       <c r="M7" s="2" t="n"/>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>Gien Faience</t>
-        </is>
-      </c>
-      <c r="O7" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P7" s="2" t="n">
-        <v>3.747</v>
-      </c>
+      <c r="N7" s="2" t="n"/>
+      <c r="O7" s="2" t="n"/>
+      <c r="P7" s="2" t="n"/>
       <c r="Q7" s="2" t="n"/>
-      <c r="R7" s="2" t="inlineStr">
-        <is>
-          <t>Majolica</t>
-        </is>
-      </c>
-      <c r="S7" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="T7" s="2" t="n">
-        <v>1.802</v>
-      </c>
+      <c r="R7" s="2" t="n"/>
+      <c r="S7" s="2" t="n"/>
+      <c r="T7" s="2" t="n"/>
       <c r="U7" s="2" t="n"/>
-      <c r="V7" s="2" t="inlineStr">
-        <is>
-          <t>Gien Faience</t>
-        </is>
-      </c>
-      <c r="W7" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="X7" s="2" t="n">
-        <v>25.087</v>
-      </c>
+      <c r="V7" s="2" t="n"/>
+      <c r="W7" s="2" t="n"/>
+      <c r="X7" s="2" t="n"/>
       <c r="Y7" s="2" t="n"/>
     </row>
     <row r="8" ht="58" customHeight="1">
@@ -5288,62 +5096,30 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Jingdezhen</t>
+          <t>Bat Trang ceramics</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I8" s="2" t="n"/>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>Jingdezhen</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="L8" s="2" t="n">
-        <v>8.114000000000001</v>
-      </c>
+      <c r="J8" s="2" t="n"/>
+      <c r="K8" s="2" t="n"/>
+      <c r="L8" s="2" t="n"/>
       <c r="M8" s="2" t="n"/>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>Jingdezhen</t>
-        </is>
-      </c>
-      <c r="O8" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P8" s="2" t="n">
-        <v>4.496</v>
-      </c>
+      <c r="N8" s="2" t="n"/>
+      <c r="O8" s="2" t="n"/>
+      <c r="P8" s="2" t="n"/>
       <c r="Q8" s="2" t="n"/>
-      <c r="R8" s="2" t="inlineStr">
-        <is>
-          <t>Jingdezhen</t>
-        </is>
-      </c>
-      <c r="S8" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T8" s="2" t="n">
-        <v>2.305</v>
-      </c>
+      <c r="R8" s="2" t="n"/>
+      <c r="S8" s="2" t="n"/>
+      <c r="T8" s="2" t="n"/>
       <c r="U8" s="2" t="n"/>
-      <c r="V8" s="2" t="inlineStr">
-        <is>
-          <t>Jingdezhen</t>
-        </is>
-      </c>
-      <c r="W8" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="X8" s="2" t="n">
-        <v>21.801</v>
-      </c>
+      <c r="V8" s="2" t="n"/>
+      <c r="W8" s="2" t="n"/>
+      <c r="X8" s="2" t="n"/>
       <c r="Y8" s="2" t="n"/>
     </row>
     <row r="9" ht="58" customHeight="1">
@@ -5373,62 +5149,30 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Jingdezhen</t>
+          <t>Bat Trang ceramics</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I9" s="2" t="n"/>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>Jingdezhen</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="L9" s="2" t="n">
-        <v>8.468999999999999</v>
-      </c>
+      <c r="J9" s="2" t="n"/>
+      <c r="K9" s="2" t="n"/>
+      <c r="L9" s="2" t="n"/>
       <c r="M9" s="2" t="n"/>
-      <c r="N9" s="2" t="inlineStr">
-        <is>
-          <t>Jingdezhen</t>
-        </is>
-      </c>
-      <c r="O9" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P9" s="2" t="n">
-        <v>4.315</v>
-      </c>
+      <c r="N9" s="2" t="n"/>
+      <c r="O9" s="2" t="n"/>
+      <c r="P9" s="2" t="n"/>
       <c r="Q9" s="2" t="n"/>
-      <c r="R9" s="2" t="inlineStr">
-        <is>
-          <t>Jingdezhen</t>
-        </is>
-      </c>
-      <c r="S9" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T9" s="2" t="n">
-        <v>1.897</v>
-      </c>
+      <c r="R9" s="2" t="n"/>
+      <c r="S9" s="2" t="n"/>
+      <c r="T9" s="2" t="n"/>
       <c r="U9" s="2" t="n"/>
-      <c r="V9" s="2" t="inlineStr">
-        <is>
-          <t>Jingdezhen</t>
-        </is>
-      </c>
-      <c r="W9" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="X9" s="2" t="n">
-        <v>27.586</v>
-      </c>
+      <c r="V9" s="2" t="n"/>
+      <c r="W9" s="2" t="n"/>
+      <c r="X9" s="2" t="n"/>
       <c r="Y9" s="2" t="n"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update ACIS specialists prompts and final Excel report
</commit_message>
<xml_diff>
--- a/outputs/gom_experiment_benchmark_report.xlsx
+++ b/outputs/gom_experiment_benchmark_report.xlsx
@@ -1380,25 +1380,25 @@
         <v>5</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>25</v>
+        <v>35.71</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>28.57</v>
+        <v>35.71</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>26.19</v>
+        <v>35.71</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>14.922</v>
+        <v>30.914</v>
       </c>
       <c r="K5" s="5" t="n">
         <v>0</v>
@@ -1419,25 +1419,25 @@
         <v>5</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E6" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>25</v>
+        <v>35.71</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>28.57</v>
+        <v>35.71</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>26.19</v>
+        <v>35.71</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>9.35</v>
+        <v>10.79</v>
       </c>
       <c r="K6" s="5" t="n">
         <v>0</v>
@@ -1458,25 +1458,25 @@
         <v>5</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>25</v>
+        <v>35.71</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>28.57</v>
+        <v>35.71</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>26.19</v>
+        <v>35.71</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>5.873</v>
+        <v>6.83</v>
       </c>
       <c r="K7" s="5" t="n">
         <v>0</v>
@@ -1497,25 +1497,25 @@
         <v>5</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>25</v>
+        <v>35.71</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>28.57</v>
+        <v>35.71</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>26.19</v>
+        <v>35.71</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>31.179</v>
+        <v>57.092</v>
       </c>
       <c r="K8" s="5" t="n">
         <v>0</v>
@@ -1539,7 +1539,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F9" s="5" t="n">
         <v>0</v>
@@ -1554,10 +1554,10 @@
         <v>0</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>13.102</v>
+        <v>41.475</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1575,28 +1575,28 @@
         <v>5</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>0</v>
+        <v>17.86</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0</v>
+        <v>21.43</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0</v>
+        <v>19.05</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>9.488</v>
+        <v>10.948</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11">
@@ -1614,28 +1614,28 @@
         <v>5</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>0</v>
+        <v>21.43</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>0</v>
+        <v>21.43</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>0</v>
+        <v>21.43</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>6.684</v>
+        <v>35.955</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -1653,28 +1653,28 @@
         <v>5</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E12" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>0</v>
+        <v>21.43</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0</v>
+        <v>21.43</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0</v>
+        <v>21.43</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>39.006</v>
+        <v>74.642</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1854,10 +1854,10 @@
         <v>5</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="F5" s="6" t="n">
         <v>0</v>
@@ -1872,19 +1872,19 @@
         <v>0</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>25</v>
+        <v>35.71</v>
       </c>
       <c r="L5" s="5" t="n">
-        <v>28.57</v>
+        <v>35.71</v>
       </c>
       <c r="M5" s="5" t="n">
-        <v>26.19</v>
+        <v>35.71</v>
       </c>
       <c r="N5" s="5" t="n">
-        <v>14.922</v>
+        <v>30.914</v>
       </c>
     </row>
     <row r="6">
@@ -1902,10 +1902,10 @@
         <v>5</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="F6" s="6" t="n">
         <v>0</v>
@@ -1920,19 +1920,19 @@
         <v>0</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>25</v>
+        <v>35.71</v>
       </c>
       <c r="L6" s="5" t="n">
-        <v>28.57</v>
+        <v>35.71</v>
       </c>
       <c r="M6" s="5" t="n">
-        <v>26.19</v>
+        <v>35.71</v>
       </c>
       <c r="N6" s="5" t="n">
-        <v>9.35</v>
+        <v>10.79</v>
       </c>
     </row>
     <row r="7">
@@ -1950,10 +1950,10 @@
         <v>5</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="F7" s="6" t="n">
         <v>0</v>
@@ -1968,19 +1968,19 @@
         <v>0</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>25</v>
+        <v>35.71</v>
       </c>
       <c r="L7" s="5" t="n">
-        <v>28.57</v>
+        <v>35.71</v>
       </c>
       <c r="M7" s="5" t="n">
-        <v>26.19</v>
+        <v>35.71</v>
       </c>
       <c r="N7" s="5" t="n">
-        <v>5.873</v>
+        <v>6.83</v>
       </c>
     </row>
     <row r="8">
@@ -1998,10 +1998,10 @@
         <v>5</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="F8" s="6" t="n">
         <v>0</v>
@@ -2016,19 +2016,19 @@
         <v>0</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>25</v>
+        <v>35.71</v>
       </c>
       <c r="L8" s="5" t="n">
-        <v>28.57</v>
+        <v>35.71</v>
       </c>
       <c r="M8" s="5" t="n">
-        <v>26.19</v>
+        <v>35.71</v>
       </c>
       <c r="N8" s="5" t="n">
-        <v>31.179</v>
+        <v>57.092</v>
       </c>
     </row>
     <row r="9">
@@ -2052,16 +2052,16 @@
         <v>0</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="J9" s="5" t="n">
         <v>0</v>
@@ -2076,7 +2076,7 @@
         <v>0</v>
       </c>
       <c r="N9" s="5" t="n">
-        <v>13.102</v>
+        <v>41.475</v>
       </c>
     </row>
     <row r="10">
@@ -2094,10 +2094,10 @@
         <v>5</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F10" s="6" t="n">
         <v>0</v>
@@ -2106,25 +2106,25 @@
         <v>0</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>0</v>
+        <v>17.86</v>
       </c>
       <c r="L10" s="5" t="n">
-        <v>0</v>
+        <v>21.43</v>
       </c>
       <c r="M10" s="5" t="n">
-        <v>0</v>
+        <v>19.05</v>
       </c>
       <c r="N10" s="5" t="n">
-        <v>9.488</v>
+        <v>10.948</v>
       </c>
     </row>
     <row r="11">
@@ -2142,37 +2142,37 @@
         <v>5</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>0</v>
+        <v>21.43</v>
       </c>
       <c r="L11" s="5" t="n">
-        <v>0</v>
+        <v>21.43</v>
       </c>
       <c r="M11" s="5" t="n">
-        <v>0</v>
+        <v>21.43</v>
       </c>
       <c r="N11" s="5" t="n">
-        <v>6.684</v>
+        <v>35.955</v>
       </c>
     </row>
     <row r="12">
@@ -2190,10 +2190,10 @@
         <v>5</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F12" s="6" t="n">
         <v>0</v>
@@ -2202,25 +2202,25 @@
         <v>0</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>0</v>
+        <v>21.43</v>
       </c>
       <c r="L12" s="5" t="n">
-        <v>0</v>
+        <v>21.43</v>
       </c>
       <c r="M12" s="5" t="n">
-        <v>0</v>
+        <v>21.43</v>
       </c>
       <c r="N12" s="5" t="n">
-        <v>39.006</v>
+        <v>74.642</v>
       </c>
     </row>
     <row r="13">
@@ -2318,28 +2318,28 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="C16" s="5" t="n">
         <v>40</v>
       </c>
-      <c r="C16" s="5" t="n">
-        <v>0</v>
-      </c>
       <c r="D16" s="5" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>12.5</v>
+        <v>17.86</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>14.29</v>
+        <v>17.86</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>13.1</v>
+        <v>17.86</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>14.012</v>
+        <v>36.195</v>
       </c>
       <c r="J16" s="2" t="n"/>
       <c r="K16" s="2" t="n"/>
@@ -2354,28 +2354,28 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="C17" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D17" s="5" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>12.5</v>
+        <v>26.79</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>14.29</v>
+        <v>28.57</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>13.1</v>
+        <v>27.38</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>9.419</v>
+        <v>10.869</v>
       </c>
       <c r="J17" s="2" t="n"/>
       <c r="K17" s="2" t="n"/>
@@ -2390,28 +2390,28 @@
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="C18" s="5" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D18" s="5" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>12.5</v>
+        <v>28.57</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>14.29</v>
+        <v>28.57</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>13.1</v>
+        <v>28.57</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>6.279</v>
+        <v>21.392</v>
       </c>
       <c r="J18" s="2" t="n"/>
       <c r="K18" s="2" t="n"/>
@@ -2426,28 +2426,28 @@
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="C19" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>12.5</v>
+        <v>28.57</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>14.29</v>
+        <v>28.57</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>13.1</v>
+        <v>28.57</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>35.093</v>
+        <v>65.867</v>
       </c>
       <c r="J19" s="2" t="n"/>
       <c r="K19" s="2" t="n"/>
@@ -2633,25 +2633,25 @@
         <v>5</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>25</v>
+        <v>35.71</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>28.57</v>
+        <v>35.71</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>26.19</v>
+        <v>35.71</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>14.922</v>
+        <v>30.914</v>
       </c>
       <c r="J7" s="5" t="n">
         <v>0</v>
@@ -2667,25 +2667,25 @@
         <v>5</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>25</v>
+        <v>35.71</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>28.57</v>
+        <v>35.71</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>26.19</v>
+        <v>35.71</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>9.35</v>
+        <v>10.79</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -2701,25 +2701,25 @@
         <v>5</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>25</v>
+        <v>35.71</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>28.57</v>
+        <v>35.71</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>26.19</v>
+        <v>35.71</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>5.873</v>
+        <v>6.83</v>
       </c>
       <c r="J9" s="5" t="n">
         <v>0</v>
@@ -2735,25 +2735,25 @@
         <v>5</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>25</v>
+        <v>35.71</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>28.57</v>
+        <v>35.71</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>26.19</v>
+        <v>35.71</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>31.179</v>
+        <v>57.092</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>0</v>
@@ -3569,7 +3569,7 @@
         <v>1</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>22.561</v>
+        <v>45.927</v>
       </c>
       <c r="M5" s="2" t="n"/>
       <c r="N5" s="2" t="inlineStr">
@@ -3581,7 +3581,7 @@
         <v>1</v>
       </c>
       <c r="P5" s="2" t="n">
-        <v>9.048</v>
+        <v>12.579</v>
       </c>
       <c r="Q5" s="2" t="n"/>
       <c r="R5" s="2" t="inlineStr">
@@ -3593,7 +3593,7 @@
         <v>1</v>
       </c>
       <c r="T5" s="2" t="n">
-        <v>5.88</v>
+        <v>10.516</v>
       </c>
       <c r="U5" s="2" t="n"/>
       <c r="V5" s="2" t="inlineStr">
@@ -3605,7 +3605,7 @@
         <v>1</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>38.373</v>
+        <v>75.863</v>
       </c>
       <c r="Y5" s="2" t="n"/>
     </row>
@@ -3912,7 +3912,7 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
@@ -3920,7 +3920,7 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G4" s="2" t="n"/>
       <c r="H4" s="2" t="n"/>
@@ -4004,7 +4004,7 @@
         <v>0</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E7" s="5" t="n">
         <v>0</v>
@@ -4019,10 +4019,10 @@
         <v>0</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>13.102</v>
+        <v>41.475</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -4035,28 +4035,28 @@
         <v>5</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>0</v>
+        <v>17.86</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>0</v>
+        <v>21.43</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0</v>
+        <v>19.05</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>9.488</v>
+        <v>10.948</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9">
@@ -4069,28 +4069,28 @@
         <v>5</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0</v>
+        <v>21.43</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>0</v>
+        <v>21.43</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>0</v>
+        <v>21.43</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>6.684</v>
+        <v>35.955</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -4103,28 +4103,28 @@
         <v>5</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0</v>
+        <v>21.43</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>0</v>
+        <v>21.43</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>0</v>
+        <v>21.43</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>39.006</v>
+        <v>74.642</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -4656,7 +4656,7 @@
     <col width="14" customWidth="1" min="19" max="19"/>
     <col width="14" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
-    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="11" customWidth="1" min="22" max="22"/>
     <col width="14" customWidth="1" min="23" max="23"/>
     <col width="14" customWidth="1" min="24" max="24"/>
     <col width="12" customWidth="1" min="25" max="25"/>
@@ -4916,50 +4916,50 @@
       <c r="I5" s="2" t="n"/>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Jingdezhen</t>
+          <t>Chu Dau</t>
         </is>
       </c>
       <c r="K5" s="2" t="b">
         <v>0</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>12.317</v>
+        <v>41.475</v>
       </c>
       <c r="M5" s="2" t="n"/>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>Jingdezhen</t>
+          <t>Bien Hoa</t>
         </is>
       </c>
       <c r="O5" s="2" t="b">
         <v>0</v>
       </c>
       <c r="P5" s="2" t="n">
-        <v>8.297000000000001</v>
+        <v>8.851000000000001</v>
       </c>
       <c r="Q5" s="2" t="n"/>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>Jingdezhen</t>
+          <t>Chu Dau</t>
         </is>
       </c>
       <c r="S5" s="2" t="b">
         <v>0</v>
       </c>
       <c r="T5" s="2" t="n">
-        <v>6.037</v>
+        <v>64.72</v>
       </c>
       <c r="U5" s="2" t="n"/>
       <c r="V5" s="2" t="inlineStr">
         <is>
-          <t>Jingdezhen</t>
+          <t>Chu Dau</t>
         </is>
       </c>
       <c r="W5" s="2" t="b">
         <v>0</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>26.728</v>
+        <v>112.751</v>
       </c>
       <c r="Y5" s="2" t="n"/>
     </row>

</xml_diff>